<commit_message>
Importação: legenda no modelo, colunas Autor/Réu/Tribunal, tipo Contato, e botão Manual em Configurações
- Adiciona campo Case.tribunal (sigla do tribunal, ex: TJGO, TRF1, TST)
- importCasesCore: suporta colunas Autor/Réu (identifica o cliente pelo
  Papel do cliente, mantendo compatibilidade com Cliente/Outros envolvidos)
  e o novo valor de Tipo "Contato" (cadastra só o contato, sem processo)
- Modelo .xlsx de Processos/Casos/Atendimentos ganha aba "Legenda" com
  orientações de preenchimento (formato CNJ do número do processo, como
  indicar o cliente, siglas de tribunal aceitas) e as novas colunas
  Autor, Réu e Tribunal
- Botão "Manual" em Configurações → Geral abre modal com a mesma legenda,
  estilizado em dourado e bordô
</commit_message>
<xml_diff>
--- a/public/templates/modelo-processos-casos-atendimentos.xlsx
+++ b/public/templates/modelo-processos-casos-atendimentos.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Modelo" sheetId="1" r:id="rId1"/>
+    <sheet name="Legenda" sheetId="1" r:id="rId1"/>
+    <sheet name="Modelo" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,36 +398,280 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:B33"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>LEGENDA PARA PREENCHIMENTO</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Esta aba é só de leitura — os dados de verdade ficam na aba "Modelo". Leia antes de preencher.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>1. COLUNA "Tipo" — o que cada valor faz</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Valor aceito</v>
+      </c>
+      <c r="B6" t="str">
+        <v>O que acontece ao importar</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Processo</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Cria um Processo judicial (usa Número, Vara, Tribunal, Instância etc.).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Caso</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Cria um Caso (mesma estrutura de Processo, sem exigir número/tribunal).</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Atendimento</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Cria um Atendimento (consulta ou serviço avulso, sem processo).</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Contato</v>
+      </c>
+      <c r="B10" t="str">
+        <v>NÃO cria processo/caso — cadastra só o contato (Cliente/Autor/Réu preenchido) em Contatos → Clientes.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2. FORMATO DO NÚMERO DO PROCESSO (padrão CNJ)</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Máscara</v>
+      </c>
+      <c r="B13" t="str">
+        <v>NNNNNNN-DD.AAAA.J.TR.OOOO</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Exemplo preenchido</v>
+      </c>
+      <c r="B14" t="str">
+        <v>0001234-56.2026.8.09.0051</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>O que é cada parte</v>
+      </c>
+      <c r="B15" t="str">
+        <v>NNNNNNN = número sequencial do processo (7 dígitos) · DD = dígito verificador (2 dígitos) · AAAA = ano de ajuizamento (4 dígitos) · J = segmento de justiça (1 dígito, ex: 8 = Justiça Estadual) · TR = tribunal (2 dígitos) · OOOO = unidade de origem (4 dígitos)</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>3. COMO INDICAR O CLIENTE (quem é o NOSSO cliente no processo)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Forma simples (como já era)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Preencha só a coluna "Cliente" com o nome do seu cliente. "Outros envolvidos" recebe a parte contrária, se quiser registrar.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Forma recomendada (mais clara)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Preencha "Autor" e "Réu" com os nomes das partes do processo, e diga em "Papel do cliente" qual das duas é o seu cliente (ex: "Autor" ou "Réu"). O sistema identifica automaticamente quem é o cliente e quem é a parte contrária.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Se preencher Autor/Réu e Cliente juntos</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Autor/Réu tem prioridade — a coluna "Cliente" é ignorada nesse caso.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>4. SIGLAS DE TRIBUNAL ACEITAS NA COLUNA "Tribunal"</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Grupo</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Siglas</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Tribunais superiores</v>
+      </c>
+      <c r="B24" t="str">
+        <v>STF, STJ, TST, TSE, STM</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Justiça Estadual (2º grau)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>TJ + sigla do estado, ex: TJGO, TJSP, TJRJ, TJMG...</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Justiça Federal</v>
+      </c>
+      <c r="B26" t="str">
+        <v>TRF1, TRF2, TRF3, TRF4, TRF5, TRF6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Justiça do Trabalho</v>
+      </c>
+      <c r="B27" t="str">
+        <v>TRT1 a TRT24</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Justiça Eleitoral</v>
+      </c>
+      <c r="B28" t="str">
+        <v>TRE + sigla do estado, ex: TREGO, TRESP...</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>5. OUTRAS ORIENTAÇÕES</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Campos em branco</v>
+      </c>
+      <c r="B31" t="str">
+        <v>São ignorados — preencha só o que tiver.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Datas</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Formato DD/MM/AAAA (ex: 21/07/2026).</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Valores monetários</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Só números, sem "R$" e sem separador de milhar (ex: 15000 ou 15000,50).</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B33"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AE2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="17.83203125" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" customWidth="1"/>
     <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
     <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="21.83203125" customWidth="1"/>
-    <col min="16" max="16" width="21.83203125" customWidth="1"/>
-    <col min="17" max="17" width="23.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="22.83203125" customWidth="1"/>
-    <col min="21" max="21" width="26.83203125" customWidth="1"/>
-    <col min="22" max="22" width="31.83203125" customWidth="1"/>
-    <col min="23" max="23" width="20.83203125" customWidth="1"/>
-    <col min="24" max="24" width="17.83203125" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
-    <col min="26" max="26" width="12.83203125" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" customWidth="1"/>
-    <col min="28" max="28" width="13.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="21.83203125" customWidth="1"/>
+    <col min="18" max="18" width="21.83203125" customWidth="1"/>
+    <col min="19" max="19" width="23.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="17.83203125" customWidth="1"/>
+    <col min="22" max="22" width="22.83203125" customWidth="1"/>
+    <col min="23" max="23" width="26.83203125" customWidth="1"/>
+    <col min="24" max="24" width="31.83203125" customWidth="1"/>
+    <col min="25" max="25" width="20.83203125" customWidth="1"/>
+    <col min="26" max="26" width="17.83203125" customWidth="1"/>
+    <col min="27" max="27" width="17.83203125" customWidth="1"/>
+    <col min="28" max="28" width="12.83203125" customWidth="1"/>
+    <col min="29" max="29" width="12.83203125" customWidth="1"/>
+    <col min="30" max="30" width="12.83203125" customWidth="1"/>
+    <col min="31" max="31" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -443,75 +688,84 @@
         <v>Cliente</v>
       </c>
       <c r="E1" t="str">
+        <v>Autor</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Réu</v>
+      </c>
+      <c r="G1" t="str">
         <v>Outros clientes</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Outros envolvidos</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Pasta</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Ação</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Número</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Data de distribuição</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>Objeto</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>Observações</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>Matéria</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>Valor da causa</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Q1" t="str">
         <v>Valor da condenação</v>
       </c>
-      <c r="P1" t="str">
+      <c r="R1" t="str">
         <v>Decisão do processo</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="S1" t="str">
         <v>Resultado do processo</v>
       </c>
-      <c r="R1" t="str">
+      <c r="T1" t="str">
         <v>Etiquetas</v>
       </c>
-      <c r="S1" t="str">
+      <c r="U1" t="str">
         <v>Data de Criação</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Data de Encerramento</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>Data do último histórico</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
         <v>Descrição do último histórico</v>
       </c>
-      <c r="W1" t="str">
+      <c r="Y1" t="str">
         <v>Instância Original</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Z1" t="str">
         <v>Instância Atual</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AA1" t="str">
         <v>URL do Processo</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AB1" t="str">
+        <v>Tribunal</v>
+      </c>
+      <c r="AC1" t="str">
         <v>Vara</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AD1" t="str">
         <v>Foro</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AE1" t="str">
         <v>Responsável</v>
       </c>
     </row>
@@ -526,44 +780,44 @@
         <v>Autor</v>
       </c>
       <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
         <v>João da Silva</v>
       </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
       <c r="F2" t="str">
+        <v>Empresa XYZ Ltda</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>Empresa XYZ Ltda (PARTE)</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>PASTA-001</v>
       </c>
-      <c r="H2" t="str">
+      <c r="J2" t="str">
         <v>Ação de Cobrança</v>
       </c>
-      <c r="I2" t="str">
-        <v>0000000-00.2026.8.09.0051</v>
-      </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
+        <v>0001234-56.2026.8.09.0051</v>
+      </c>
+      <c r="L2" t="str">
         <v>01/02/2026</v>
       </c>
-      <c r="K2" t="str">
+      <c r="M2" t="str">
         <v>Cobrança de valores em aberto</v>
       </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
         <v>Observação livre sobre o caso</v>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v>Cível</v>
       </c>
-      <c r="N2">
+      <c r="P2">
         <v>15000</v>
       </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
       <c r="Q2" t="str">
         <v/>
       </c>
@@ -571,39 +825,48 @@
         <v/>
       </c>
       <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
         <v>01/02/2026</v>
       </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
-      <c r="U2" t="str">
-        <v/>
-      </c>
       <c r="V2" t="str">
         <v/>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
         <v>1</v>
       </c>
-      <c r="X2" t="str">
+      <c r="Z2" t="str">
         <v>1</v>
       </c>
-      <c r="Y2" t="str">
-        <v/>
-      </c>
-      <c r="Z2" t="str">
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v>TJGO</v>
+      </c>
+      <c r="AC2" t="str">
         <v>3ª Vara Cível de Goiânia</v>
       </c>
-      <c r="AA2" t="str">
+      <c r="AD2" t="str">
         <v>Goiânia</v>
       </c>
-      <c r="AB2" t="str">
+      <c r="AE2" t="str">
         <v>Jairo Rodarte</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>